<commit_message>
docs: sync specifications with the foundation code
- CLAUDE.md: conventional commits rules
- api/CLAUDE.md, implement-feature: build and test ZenGear.slnx
  explicitly (MSB1011 with docker-compose.dcproj)
- API_CONVENTIONS: /health endpoint
- DATABASE: correlation_id is the W3C trace id of the request
- Blueprint: DEC-085 personal data in security logs; Tech Stack
  health check and TimeProvider.Testing packages

Refs: DEC-085, DEC-086, DEC-093
</commit_message>
<xml_diff>
--- a/docs/product-domain-blueprint-MVP.xlsx
+++ b/docs/product-domain-blueprint-MVP.xlsx
@@ -19,7 +19,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Actors'!$A$1:$H$17</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Tech Stack'!$A$1:$E$43</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Tech Stack'!$A$1:$E$45</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Roadmap'!$A$1:$G$5</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Features'!$A$1:$K$131</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Use Cases'!$A$1:$L$140</definedName>
@@ -1244,7 +1244,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E43"/>
+  <dimension ref="A1:E45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1770,22 +1770,22 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>Background Jobs</t>
+          <t>Backend API</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>BackgroundService + PeriodicTimer</t>
+          <t>Microsoft.Extensions.Diagnostics.HealthChecks.EntityFrameworkCore</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>.NET 10</t>
+          <t>—</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>Job nền của Scheduler (A10): hủy đơn quá hạn, gửi thông báo, phát hành hóa đơn, đối soát hằng đêm</t>
+          <t>Health check kết nối database cho endpoint /health</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
@@ -1797,22 +1797,22 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>Cache</t>
+          <t>Background Jobs</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>Redis</t>
+          <t>BackgroundService + PeriodicTimer</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>.NET 10</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>Cache quyền theo Role (R-SEC-07)</t>
+          <t>Job nền của Scheduler (A10): hủy đơn quá hạn, gửi thông báo, phát hành hóa đơn, đối soát hằng đêm</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
@@ -1824,22 +1824,22 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>Database</t>
+          <t>Cache</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>PostgreSQL</t>
+          <t>Redis</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>—</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>CSDL quan hệ; cần uuidv7() native; file SQL và DBML trong DATABASE.md là đặc tả để CI đối chiếu với kết quả migration</t>
+          <t>Cache quyền theo Role (R-SEC-07)</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
@@ -1856,17 +1856,17 @@
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>btree_gist</t>
+          <t>PostgreSQL</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>18</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>Extension: exclusion constraint cho tax_rates</t>
+          <t>CSDL quan hệ; cần uuidv7() native; file SQL và DBML trong DATABASE.md là đặc tả để CI đối chiếu với kết quả migration</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
@@ -1883,7 +1883,7 @@
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>unaccent + pg_trgm</t>
+          <t>btree_gist</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
@@ -1893,24 +1893,24 @@
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>Extension: tìm kiếm không dấu (PDS-03)</t>
+          <t>Extension: exclusion constraint cho tax_rates</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>Phase 2</t>
+          <t>Phase 1</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>File Storage</t>
+          <t>Database</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>Firebase Storage</t>
+          <t>unaccent + pg_trgm</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
@@ -1920,24 +1920,24 @@
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>Ảnh sản phẩm, ảnh chứng từ và bằng chứng (attachments)</t>
+          <t>Extension: tìm kiếm không dấu (PDS-03)</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>Phase 1</t>
+          <t>Phase 2</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>External Service</t>
+          <t>File Storage</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>Firebase Authentication</t>
+          <t>Firebase Storage</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
@@ -1947,7 +1947,7 @@
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>Đăng nhập nhân viên; khách đăng nhập email, Google, SĐT + OTP ở Phase 2 cần gói Blaze (A13)</t>
+          <t>Ảnh sản phẩm, ảnh chứng từ và bằng chứng (attachments)</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
@@ -1964,7 +1964,7 @@
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>Resend</t>
+          <t>Firebase Authentication</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
@@ -1974,7 +1974,7 @@
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>Gửi email giao dịch (A14)</t>
+          <t>Đăng nhập nhân viên; khách đăng nhập email, Google, SĐT + OTP ở Phase 2 cần gói Blaze (A13)</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
@@ -1991,7 +1991,7 @@
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>MISA meInvoice</t>
+          <t>Resend</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
@@ -2001,7 +2001,7 @@
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>Phát hành hóa đơn bán hàng điện tử qua API tích hợp dành cho developer (A15)</t>
+          <t>Gửi email giao dịch (A14)</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
@@ -2018,7 +2018,7 @@
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>VNPay</t>
+          <t>MISA meInvoice</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
@@ -2028,24 +2028,24 @@
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>Cổng thanh toán, dùng sandbox cho demo (A12)</t>
+          <t>Phát hành hóa đơn bán hàng điện tử qua API tích hợp dành cho developer (A15)</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>Phase 2</t>
+          <t>Phase 1</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>Testing</t>
+          <t>External Service</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>NUnit</t>
+          <t>VNPay</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
@@ -2055,12 +2055,12 @@
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>Test framework cho unit test và integration test</t>
+          <t>Cổng thanh toán, dùng sandbox cho demo (A12)</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>Phase 1</t>
+          <t>Phase 2</t>
         </is>
       </c>
     </row>
@@ -2072,7 +2072,7 @@
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>Shouldly</t>
+          <t>NUnit</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
@@ -2082,7 +2082,7 @@
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>Assertion</t>
+          <t>Test framework cho unit test và integration test</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
@@ -2099,7 +2099,7 @@
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>Moq</t>
+          <t>Shouldly</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
@@ -2109,7 +2109,7 @@
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>Mock dependency trong unit test</t>
+          <t>Assertion</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
@@ -2126,17 +2126,17 @@
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>Testcontainers for .NET</t>
+          <t>Moq</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>image postgres:18</t>
+          <t>—</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>PostgreSQL thật cho integration, concurrency và DB constraint test</t>
+          <t>Mock dependency trong unit test</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
@@ -2153,17 +2153,17 @@
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>Respawn</t>
+          <t>Testcontainers for .NET</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>image postgres:18</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>Reset dữ liệu database giữa các integration test</t>
+          <t>PostgreSQL thật cho integration, concurrency và DB constraint test</t>
         </is>
       </c>
       <c r="E34" s="2" t="inlineStr">
@@ -2180,7 +2180,7 @@
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>zengear_07_schema_check.sql</t>
+          <t>Respawn</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
@@ -2190,7 +2190,7 @@
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>Kiểm tra đủ đối tượng không có trên ERD sau mỗi migration</t>
+          <t>Reset dữ liệu database giữa các integration test</t>
         </is>
       </c>
       <c r="E35" s="2" t="inlineStr">
@@ -2202,12 +2202,12 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>Dev Tooling</t>
+          <t>Testing</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>Visual Studio / VS Code</t>
+          <t>Microsoft.Extensions.TimeProvider.Testing</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
@@ -2217,7 +2217,7 @@
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>IDE</t>
+          <t>FakeTimeProvider: điều khiển thời gian trong test của clock service (R-TZ-01)</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr">
@@ -2229,12 +2229,12 @@
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>Dev Tooling</t>
+          <t>Testing</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>pgAdmin</t>
+          <t>zengear_07_schema_check.sql</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
@@ -2244,7 +2244,7 @@
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>PostgreSQL GUI</t>
+          <t>Kiểm tra đủ đối tượng không có trên ERD sau mỗi migration</t>
         </is>
       </c>
       <c r="E37" s="2" t="inlineStr">
@@ -2261,7 +2261,7 @@
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>Postman</t>
+          <t>Visual Studio / VS Code</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
@@ -2271,7 +2271,7 @@
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>API testing</t>
+          <t>IDE</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr">
@@ -2288,7 +2288,7 @@
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>Firebase Local Emulator Suite</t>
+          <t>pgAdmin</t>
         </is>
       </c>
       <c r="C39" s="2" t="inlineStr">
@@ -2298,7 +2298,7 @@
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>Chạy Firebase local</t>
+          <t>PostgreSQL GUI</t>
         </is>
       </c>
       <c r="E39" s="2" t="inlineStr">
@@ -2315,17 +2315,17 @@
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>Docker</t>
+          <t>Postman</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>image postgres:18</t>
+          <t>—</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>Container local, khớp version Azure Database for PostgreSQL</t>
+          <t>API testing</t>
         </is>
       </c>
       <c r="E40" s="2" t="inlineStr">
@@ -2337,12 +2337,12 @@
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>Source &amp; Docs</t>
+          <t>Dev Tooling</t>
         </is>
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>Git + GitHub</t>
+          <t>Firebase Local Emulator Suite</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
@@ -2352,7 +2352,7 @@
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>Quản lý mã nguồn; một repository cho api, web và docs (DEC-093)</t>
+          <t>Chạy Firebase local</t>
         </is>
       </c>
       <c r="E41" s="2" t="inlineStr">
@@ -2364,22 +2364,22 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>Source &amp; Docs</t>
+          <t>Dev Tooling</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>GitHub Actions</t>
+          <t>Docker</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>image postgres:18</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>CI theo path filter: api.yml build, test, kiểm tra migration; web.yml build web và so kiểu dữ liệu sinh từ OpenAPI (DEC-093)</t>
+          <t>Container local, khớp version Azure Database for PostgreSQL</t>
         </is>
       </c>
       <c r="E42" s="2" t="inlineStr">
@@ -2396,27 +2396,81 @@
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
+          <t>Git + GitHub</t>
+        </is>
+      </c>
+      <c r="C43" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D43" s="2" t="inlineStr">
+        <is>
+          <t>Quản lý mã nguồn; một repository cho api, web và docs (DEC-093)</t>
+        </is>
+      </c>
+      <c r="E43" s="2" t="inlineStr">
+        <is>
+          <t>Phase 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>Source &amp; Docs</t>
+        </is>
+      </c>
+      <c r="B44" s="2" t="inlineStr">
+        <is>
+          <t>GitHub Actions</t>
+        </is>
+      </c>
+      <c r="C44" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D44" s="2" t="inlineStr">
+        <is>
+          <t>CI theo path filter: api.yml build, test, kiểm tra migration; web.yml build web và so kiểu dữ liệu sinh từ OpenAPI (DEC-093)</t>
+        </is>
+      </c>
+      <c r="E44" s="2" t="inlineStr">
+        <is>
+          <t>Phase 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="2" t="inlineStr">
+        <is>
+          <t>Source &amp; Docs</t>
+        </is>
+      </c>
+      <c r="B45" s="2" t="inlineStr">
+        <is>
           <t>dbdocs.io</t>
         </is>
       </c>
-      <c r="C43" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D43" s="2" t="inlineStr">
+      <c r="C45" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D45" s="2" t="inlineStr">
         <is>
           <t>Tài liệu ERD sinh từ khối DBML trong DATABASE.md</t>
         </is>
       </c>
-      <c r="E43" s="2" t="inlineStr">
+      <c r="E45" s="2" t="inlineStr">
         <is>
           <t>Phase 1</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E43"/>
+  <autoFilter ref="A1:E45"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -33870,7 +33924,7 @@
       </c>
       <c r="E86" s="2" t="inlineStr">
         <is>
-          <t>Không có màn hình xem lịch sử đăng nhập trong ứng dụng; thời hạn lưu cấu hình ở nơi lưu log. Khi có feature Lịch sử đăng nhập thì thêm bảng user_login_events (một dòng mỗi auth_time); khi cần đăng xuất theo từng thiết bị thì thêm user_sessions; khi cần màn hình nhật ký hoạt động nhân viên thì thêm VIEW ghép hai nguồn, lọc quyền theo nguồn ở API.</t>
+          <t>Không có màn hình xem lịch sử đăng nhập trong ứng dụng; thời hạn lưu cấu hình ở nơi lưu log. Log bảo mật chứa IP và user agent là dữ liệu cá nhân, nên nơi lưu log phải giới hạn quyền đọc và có thời hạn xóa như dữ liệu cá nhân khác. Khi có feature Lịch sử đăng nhập thì thêm bảng user_login_events (một dòng mỗi auth_time); khi cần đăng xuất theo từng thiết bị thì thêm user_sessions; khi cần màn hình nhật ký hoạt động nhân viên thì thêm VIEW ghép hai nguồn, lọc quyền theo nguồn ở API.</t>
         </is>
       </c>
       <c r="F86" s="2" t="inlineStr">

</xml_diff>

<commit_message>
docs: decide how staff change passwords (DEC-094)
- Blueprint: DEC-094 password change through the API with Firebase
  Admin SDK, recent sign-in (auth_time within 5 minutes), clear
  must_change_password, revoke refresh tokens; R-USR-03, R-USR-04,
  STF-03 and UC-007 updated
- API_CONVENTIONS: /problems/recent-login-required
- implement-feature: implementation rules live in technical-design.md

Refs: DEC-094, R-USR-03, R-USR-04, STF-03
</commit_message>
<xml_diff>
--- a/docs/product-domain-blueprint-MVP.xlsx
+++ b/docs/product-domain-blueprint-MVP.xlsx
@@ -25,7 +25,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Use Cases'!$A$1:$L$140</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Domain Model'!$A$1:$J$78</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Business Rules'!$A$1:$I$134</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Decisions'!$A$1:$H$94</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Decisions'!$A$1:$H$95</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Technical Design'!$A$1:$E$17</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -3261,7 +3261,8 @@
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>- Chỉ sửa được tên hiển thị và đổi mật khẩu qua Firebase.
+          <t>- Chỉ sửa được tên hiển thị và đổi mật khẩu.
+- Đổi mật khẩu qua API bằng Firebase Admin SDK, chỉ khi lần đăng nhập gần nhất trong 5 phút; thành công thì xóa must_change_password và thu hồi các phiên khác (R-USR-03, R-USR-04, DEC-094).
 - Nhân viên không tự sửa email (@company, định danh đăng nhập, set lúc STF-01); Admin đổi khi cần (R-USR-04).
 - SĐT công việc lưu ở StaffProfile.work_phone.</t>
         </is>
@@ -11071,18 +11072,19 @@
         <is>
           <t>1. Sales Consultant mở trang tài khoản cá nhân.
 2. Sales Consultant sửa tên hiển thị hoặc chọn đổi mật khẩu.
-3. Hệ thống lưu tên hiển thị; đổi mật khẩu thực hiện qua Firebase.
+3. Hệ thống lưu tên hiển thị; đổi mật khẩu qua Firebase Admin SDK, xóa must_change_password và thu hồi các phiên khác (R-USR-04).
 4. Hệ thống hiển thị thông tin tài khoản đã cập nhật.</t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>2a. Nhân viên muốn sửa email: hệ thống không cho sửa; Admin đổi trong quản lý tài khoản nhân viên (R-USR-04).</t>
+          <t>2a. Nhân viên muốn sửa email: hệ thống không cho sửa; Admin đổi trong quản lý tài khoản nhân viên (R-USR-04).
+3a. Lần đăng nhập gần nhất quá 5 phút: hệ thống yêu cầu đăng nhập lại rồi đổi mật khẩu (DEC-094).</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>Tên hiển thị hoặc mật khẩu của nhân viên được cập nhật.</t>
+          <t>Tên hiển thị hoặc mật khẩu của nhân viên được cập nhật; sau khi đổi mật khẩu, cờ must_change_password được xóa và các phiên khác phải đăng nhập lại.</t>
         </is>
       </c>
       <c r="K8" s="2" t="inlineStr">
@@ -24909,7 +24911,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>ACTIVE ↔ DISABLED; ANONYMIZED là trạng thái cuối, không đảo ngược; Staff có must_change_password = true phải đổi mật khẩu trước khi dùng chức năng khác; ẩn danh hóa xóa gender, date_of_birth, phone, phone_verified_at, tắt marketing_consent và xóa marketing_consent_at/source/version trong customer_profiles; dữ liệu cá nhân trong audit_logs và notifications xóa theo R-USR-09</t>
+          <t>ACTIVE ↔ DISABLED; ANONYMIZED là trạng thái cuối, không đảo ngược; Staff có must_change_password = true phải đổi mật khẩu trước khi dùng chức năng khác; cờ must_change_password chỉ được xóa khi đổi mật khẩu thành công qua API (DEC-094); ẩn danh hóa xóa gender, date_of_birth, phone, phone_verified_at, tắt marketing_consent và xóa marketing_consent_at/source/version trong customer_profiles; dữ liệu cá nhân trong audit_logs và notifications xóa theo R-USR-09</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
@@ -24929,7 +24931,7 @@
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>DEC-048; DEC-022</t>
+          <t>DEC-048; DEC-022; DEC-094</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
@@ -24956,7 +24958,7 @@
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>Customer (ACC-01) sửa được tên hiển thị và hồ sơ tùy chọn (giới tính, ngày sinh, đồng ý marketing); Staff (STF-03) chỉ sửa tên hiển thị; đổi mật khẩu qua Firebase; đổi email: khách đăng nhập lại, Firebase gửi link xác nhận tới email mới, chỉ cập nhật users.email khi link được xác nhận; email mới không trùng tài khoản khác, chữ thường; ghi audit_logs và thông báo tới email cũ; email nhân viên do Admin đổi trong quản lý tài khoản nhân viên (STF-01); gộp placeholder (AUT-07, R-SEC-08) chỉ dùng email đã xác minh; SĐT tài khoản chỉ thêm/đổi sau khi xác minh OTP qua Firebase, không trùng tài khoản khác</t>
+          <t>Customer (ACC-01) sửa được tên hiển thị và hồ sơ tùy chọn (giới tính, ngày sinh, đồng ý marketing); Staff (STF-03) chỉ sửa tên hiển thị; đổi mật khẩu qua API ZenGear bằng Firebase Admin SDK, chỉ nhận khi lần đăng nhập gần nhất trong 5 phút và thu hồi các phiên khác sau khi đổi (DEC-094); đổi email: khách đăng nhập lại, Firebase gửi link xác nhận tới email mới, chỉ cập nhật users.email khi link được xác nhận; email mới không trùng tài khoản khác, chữ thường; ghi audit_logs và thông báo tới email cũ; email nhân viên do Admin đổi trong quản lý tài khoản nhân viên (STF-01); gộp placeholder (AUT-07, R-SEC-08) chỉ dùng email đã xác minh; SĐT tài khoản chỉ thêm/đổi sau khi xác minh OTP qua Firebase, không trùng tài khoản khác</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
@@ -24976,7 +24978,7 @@
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>DEC-019; DEC-053</t>
+          <t>DEC-019; DEC-053; DEC-094</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
@@ -30318,7 +30320,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H94"/>
+  <dimension ref="A1:H95"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -34279,8 +34281,50 @@
         </is>
       </c>
     </row>
+    <row r="95">
+      <c r="A95" s="2" t="inlineStr">
+        <is>
+          <t>DEC-094</t>
+        </is>
+      </c>
+      <c r="B95" s="2" t="inlineStr">
+        <is>
+          <t>Đổi mật khẩu và xóa cờ must_change_password</t>
+        </is>
+      </c>
+      <c r="C95" s="2" t="inlineStr">
+        <is>
+          <t>Nhân viên mới dùng chung mật khẩu mặc định từ biến môi trường (STF-01); cờ must_change_password là cơ chế duy nhất buộc thay mật khẩu đó (R-USR-03). Nếu web tự đổi mật khẩu qua Firebase rồi báo API xóa cờ, API không kiểm chứng được mật khẩu đã đổi.</t>
+        </is>
+      </c>
+      <c r="D95" s="2" t="inlineStr">
+        <is>
+          <t>Mọi lần đổi mật khẩu (bắt buộc và tự đổi ở STF-03) đi qua một endpoint của API: API chỉ nhận khi auth_time của ID token trong 5 phút gần nhất (nếu không trả 403 /problems/recent-login-required để web đăng nhập lại), đổi mật khẩu bằng Firebase Admin SDK sau IAuthProvider, xóa must_change_password và ghi audit_logs, rồi thu hồi refresh token (revokeRefreshTokens). Không chọn: web đổi qua Firebase rồi báo API (không kiểm chứng được); gửi link đặt mật khẩu thay mật khẩu mặc định (thay quyết định của STF-01, xem lại khi làm STF-01).</t>
+        </is>
+      </c>
+      <c r="E95" s="2" t="inlineStr">
+        <is>
+          <t>Mật khẩu đi qua API trên HTTPS và không bao giờ được ghi log (R-SEC-11). Firebase đổi trước, DB sau: lỗi ở DB chỉ khiến cờ còn nguyên và nhân viên đổi lại, không bao giờ cờ bị xóa khi mật khẩu chưa đổi. Các thiết bị đã đăng nhập bằng mật khẩu cũ bị đăng xuất; lần đăng nhập mới được ghi theo R-SEC-11. Chính sách độ mạnh mật khẩu chưa quy định, chốt khi làm STF-03.</t>
+        </is>
+      </c>
+      <c r="F95" s="2" t="inlineStr">
+        <is>
+          <t>Firebase — Manage Session Cookies (kiểm tra auth_time trong 5 phút); Firebase — Manage User Sessions (revokeRefreshTokens)</t>
+        </is>
+      </c>
+      <c r="G95" s="2" t="inlineStr">
+        <is>
+          <t>Phase 1</t>
+        </is>
+      </c>
+      <c r="H95" s="2" t="inlineStr">
+        <is>
+          <t>Accepted</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:H94"/>
+  <autoFilter ref="A1:H95"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
chore(docs): decide system roles, default roles and permission sync (DEC-095)
- Blueprint: DEC-095; AUT-04 and AUT-05 acceptance criteria (9 seeded roles, only Admin and Customer are system roles, default roles keep the Admin's edits and cannot be renamed or deleted)
- Tech Stack: StackExchange.Redis, Testcontainers Redis

Refs: DEC-095, AUT-04, AUT-05
</commit_message>
<xml_diff>
--- a/docs/product-domain-blueprint-MVP.xlsx
+++ b/docs/product-domain-blueprint-MVP.xlsx
@@ -25,7 +25,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Use Cases'!$A$1:$L$140</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Domain Model'!$A$1:$J$78</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Business Rules'!$A$1:$I$134</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Decisions'!$A$1:$H$95</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Decisions'!$A$1:$H$96</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Technical Design'!$A$1:$E$17</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1829,7 +1829,7 @@
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>Redis</t>
+          <t>Redis + StackExchange.Redis</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
@@ -1839,7 +1839,7 @@
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>Cache quyền theo Role (R-SEC-07)</t>
+          <t>Cache trạng thái user và quyền theo Role với key có phiên bản (R-SEC-07); maxmemory-policy volatile-* hoặc noeviction</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
@@ -2158,12 +2158,12 @@
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>image postgres:18</t>
+          <t>image postgres:18, redis</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>PostgreSQL thật cho integration, concurrency và DB constraint test</t>
+          <t>PostgreSQL và Redis thật cho integration, concurrency, DB constraint và cache test</t>
         </is>
       </c>
       <c r="E34" s="2" t="inlineStr">
@@ -2906,7 +2906,9 @@
           <t>- Middleware kiểm tra Permission qua Role trước mọi request.
 - scoping_type chỉ nhận 2 giá trị NONE/SELF.
 - Role có is_system_role=true (Admin, Customer) không cho sửa Permission qua UI/API.
-- Cần cache (Redis) để tránh JOIN nhiều bảng mỗi request; có thể chưa implement ở bản demo.</t>
+- Mọi endpoint khai báo quyền truy cập (permission, người dùng đã đăng ký hoặc công khai); thiếu quyền trả 403 /problems/permission-denied.
+- Cache trạng thái user và quyền theo Role trong Redis (R-SEC-07); thay đổi có hiệu lực ở request kế tiếp.
+- Danh mục permission và quyền mặc định định nghĩa trong code, đồng bộ lúc khởi động (DEC-095).</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
@@ -2965,7 +2967,8 @@
         <is>
           <t>- Chỉ Admin được thao tác.
 - Xóa Role đang gán cho Staff bị từ chối.
-- Seed sẵn 8 Role: Admin, Store Manager, Sales Consultant, Technical Support, Cashier, Warehouse Keeper, Purchasing, Customer.
+- Seed sẵn 9 Role: Admin, Store Manager, Sales Consultant, Technical Support, Cashier, Warehouse Keeper, Purchasing, Accountant, Customer.
+- 7 Role mặc định (trừ Admin, Customer) nhận quyền mặc định từ code; Admin sửa được quyền của chúng; không đổi tên, không xóa Role mặc định (DEC-095).
 - Role có is_system_role=true (Admin, Customer) không cho sửa/xóa Permission.
 - Cấu hình max_discount_percent cho từng Role (giảm giá thủ công tối đa tại quầy); NULL = không được giảm (PRM-04).</t>
         </is>
@@ -30320,7 +30323,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H95"/>
+  <dimension ref="A1:H96"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -34323,8 +34326,50 @@
         </is>
       </c>
     </row>
+    <row r="96">
+      <c r="A96" s="2" t="inlineStr">
+        <is>
+          <t>DEC-095</t>
+        </is>
+      </c>
+      <c r="B96" s="2" t="inlineStr">
+        <is>
+          <t>Role hệ thống, Role mặc định và danh mục permission</t>
+        </is>
+      </c>
+      <c r="C96" s="2" t="inlineStr">
+        <is>
+          <t>AUT-04, AUT-05 ghi Admin và Customer là Role hệ thống, trong khi seed đánh dấu cả 9 Role là hệ thống; AUT-05 yêu cầu Admin tự phân quyền không cần sửa code. Permission (resource.action) gắn với endpoint nên phải có trong code.</t>
+        </is>
+      </c>
+      <c r="D96" s="2" t="inlineStr">
+        <is>
+          <t>Danh mục permission và quyền mặc định của mỗi Role định nghĩa trong code, đồng bộ vào permissions/role_permissions lúc API khởi động (một transaction, advisory lock). Chỉ Admin và Customer là Role hệ thống (is_system_role = true): quyền luôn bị ghi đè đúng theo code, không sửa qua UI/API. 7 Role còn lại là Role mặc định (is_system_role = false): chỉ được cấp các permission key mới xuất hiện theo danh sách mặc định, không bị thu hồi hay cấp lại key đã có, nên chỉnh sửa của Admin (AUT-05) được giữ. Thiếu bất kỳ Role nào trong danh mục thì đồng bộ không ghi gì.</t>
+        </is>
+      </c>
+      <c r="E96" s="2" t="inlineStr">
+        <is>
+          <t>Thứ tự deploy: migration → zengear_08_roles.sql → seed → khởi động API. Role mặc định không được đổi tên hay xóa (đồng bộ tìm Role theo tên). Thêm một key đã có vào danh sách mặc định của Role không tự áp dụng cho database đang chạy, cần data migration. Key bị bỏ khỏi code bị xóa cùng các quyền đã gán (ghi log cảnh báo). Đồng bộ lỗi thì giữ quyền cũ, permission mới bị từ chối.</t>
+        </is>
+      </c>
+      <c r="F96" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G96" s="2" t="inlineStr">
+        <is>
+          <t>Phase 1</t>
+        </is>
+      </c>
+      <c r="H96" s="2" t="inlineStr">
+        <is>
+          <t>Accepted</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:H95"/>
+  <autoFilter ref="A1:H96"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
docs: record DEC-096 for the first admin account
Only an Admin creates staff and grants the Admin role (STF-01,
R-TX-11), and R-SEC-02 keeps at least one Admin, so each environment
needs its first Admin exactly once. The seed left this open.

DEC-096: a one-off bootstrap-admin command of ZenGear.Api, run by the
operator on the target environment. It refuses when an Admin exists,
finds or creates the Firebase user through IAuthProvider, creates the
user, staff profile and Admin role in one transaction and prints a
password reset link to the terminal only. A configured admin email
granted at first sign-in, hand-written SQL and first-user-is-admin
were rejected.

The seed README points to the command, and docs/ARCHITECTURE.md
places one-off host commands in ZenGear.Api/Hosting.

Refs: DEC-096, STF-01
</commit_message>
<xml_diff>
--- a/docs/product-domain-blueprint-MVP.xlsx
+++ b/docs/product-domain-blueprint-MVP.xlsx
@@ -25,7 +25,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Use Cases'!$A$1:$L$140</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Domain Model'!$A$1:$J$78</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Business Rules'!$A$1:$I$134</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Decisions'!$A$1:$H$97</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Decisions'!$A$1:$H$98</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Technical Design'!$A$1:$E$17</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -30323,7 +30323,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H97"/>
+  <dimension ref="A1:H98"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -34371,47 +34371,89 @@
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
         <is>
+          <t>DEC-096</t>
+        </is>
+      </c>
+      <c r="B97" s="2" t="inlineStr">
+        <is>
+          <t>Tạo tài khoản Admin đầu tiên</t>
+        </is>
+      </c>
+      <c r="C97" s="2" t="inlineStr">
+        <is>
+          <t>Chỉ Admin tạo được nhân viên và gán Role Admin (STF-01, R-TX-11), còn R-SEC-02 luôn giữ ít nhất một Admin, nên mỗi môi trường chỉ cần tạo Admin đầu tiên đúng một lần. API chỉ nhận Firebase user đã có users.firebase_uid, và seed không tạo tài khoản nào.</t>
+        </is>
+      </c>
+      <c r="D97" s="2" t="inlineStr">
+        <is>
+          <t>Lệnh một lần bootstrap-admin của ZenGear.Api (dotnet ZenGear.Api.dll bootstrap-admin --email &lt;email&gt; --name &lt;tên&gt;), do người vận hành chạy trên môi trường đích: docker compose run ở local, SSH console của Azure App Service ở production. Dưới advisory lock, lệnh từ chối nếu đã có user giữ Role Admin; lấy Firebase user theo email qua IAuthProvider, tạo mới nếu chưa có; trong một transaction tạo users (email chuẩn hóa theo R-USR-02, ACTIVE), staff_profiles (must_change_password = false) và gán Role Admin; sau khi commit in ra terminal link đặt mật khẩu (Firebase Admin SDK GeneratePasswordResetLinkAsync) để chủ cửa hàng tự đặt mật khẩu, và ghi một dòng log có cấu trúc chỉ với user_id. Không chọn: email Admin trong cấu hình, nhận quyền ở lần đăng nhập đầu (pipeline đăng nhập luôn có một nhánh cấp quyền cao nhất dựa vào claim email_verified); chèn SQL tay (chép firebase_uid, không kiểm tra gì, chạy bằng schema owner); người đăng ký đầu tiên thành Admin (ai tới API trước chiếm quyền).</t>
+        </is>
+      </c>
+      <c r="E97" s="2" t="inlineStr">
+        <is>
+          <t>Làm cùng STF-01, dùng chung IAuthProvider (ZenGear.Data/Externals/Auth) và cách tạo tài khoản nhân viên của area Identity; lớp đọc lệnh nằm ở ZenGear.Api/Hosting. Chạy lại khi đã có Admin chỉ báo lỗi, không thay đổi gì. Link đặt mật khẩu là thông tin đăng nhập: chỉ in ra terminal của người chạy lệnh, không ghi vào log, hết hạn theo Firebase. Admin tự đặt mật khẩu nên không chờ STF-03; nhân viên do STF-01 tạo dùng mật khẩu mặc định và bị chặn ở các endpoint được bảo vệ cho tới khi có endpoint đổi mật khẩu của STF-03 (DEC-094), nên làm STF-03 ngay sau STF-01.</t>
+        </is>
+      </c>
+      <c r="F97" s="2" t="inlineStr">
+        <is>
+          <t>Django — createsuperuser; Keycloak — Bootstrapping and recovering an admin account; Firebase — Generating Email Action Links</t>
+        </is>
+      </c>
+      <c r="G97" s="2" t="inlineStr">
+        <is>
+          <t>Phase 1</t>
+        </is>
+      </c>
+      <c r="H97" s="2" t="inlineStr">
+        <is>
+          <t>Accepted</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="2" t="inlineStr">
+        <is>
           <t>DEC-097</t>
         </is>
       </c>
-      <c r="B97" s="2" t="inlineStr">
+      <c r="B98" s="2" t="inlineStr">
         <is>
           <t>Cấu trúc thư mục backend</t>
         </is>
       </c>
-      <c r="C97" s="2" t="inlineStr">
+      <c r="C98" s="2" t="inlineStr">
         <is>
           <t>Code do Claude Code viết theo docs/ARCHITECTURE.md, nên mọi quy tắc cấu trúc phải kiểm được bằng test. Đã so sánh: xếp theo area trong một project (nopCommerce, Smartstore), Request/Response riêng ở Api (Bitwarden), vertical slice, mỗi area một project (GrandNode). Rủi ro ở các dự án này nằm ở service phình to (OrderProcessingService của nopCommerce 3.563 dòng) và area ghi bảng của area khác, không nằm ở cách xếp thư mục.</t>
         </is>
       </c>
-      <c r="D97" s="2" t="inlineStr">
+      <c r="D98" s="2" t="inlineStr">
         <is>
           <t>Giữ 3 project Api → Services → Data: Api xếp theo vai trò kỹ thuật; Services theo area (Models, Enums, Validators, thư mục cơ chế từ 5 type); Data theo loại rồi theo area (ARCHITECTURE.md, Folder structure). Use case nằm ở area sở hữu aggregate nó tạo hoặc thay đổi, chỉ ghi bảng của area đó và gọi service của area khác (quy tắc 4). Service tách theo nhóm use case (&lt;Entity&gt;&lt;UseCase&gt;Service), storefront dùng &lt;Entity&gt;PublicService; mỗi file của Services tối đa 400 dòng code, mỗi *Service tối đa 10 public method. Tên type không trùng trong 3 project, không có type public lồng nhau. ZenGear.ArchitectureTests kiểm các quy tắc này. Không chọn: Request/Response riêng ở Api (4 model và 3 lần map cho mỗi use case khi chưa có host thứ hai); vertical slice (DTO dùng cho nhiều use case không có chỗ duy nhất); mỗi area một project (trái với một ZenGearDbContext và một transaction xuyên area); Clean Architecture.</t>
         </is>
       </c>
-      <c r="E97" s="2" t="inlineStr">
+      <c r="E98" s="2" t="inlineStr">
         <is>
           <t>Chỉ mở lại khi tools/structure_metrics.py cho thấy: thư mục gốc của area hoặc thư mục cơ chế quá 20 file, Models/ quá 40 file, số thư mục mỗi commit feat tăng qua 3 area liên tiếp; khi test kích thước có quá 3 ngoại lệ; hoặc khi có host thứ hai dùng ZenGear.Services hay cần API phiên bản 2 (khi đó Request/Response chuyển về Api). Đổi namespace của entity làm đổi snapshot của EF Core, nên area của mỗi entity chốt trước migration của phase.</t>
         </is>
       </c>
-      <c r="F97" s="2" t="inlineStr">
+      <c r="F98" s="2" t="inlineStr">
         <is>
           <t>nopCommerce, Smartstore (area trong một project); Bitwarden (Request/Response ở Api); GrandNode (mỗi area một project)</t>
         </is>
       </c>
-      <c r="G97" s="2" t="inlineStr">
-        <is>
-          <t>Phase 1</t>
-        </is>
-      </c>
-      <c r="H97" s="2" t="inlineStr">
+      <c r="G98" s="2" t="inlineStr">
+        <is>
+          <t>Phase 1</t>
+        </is>
+      </c>
+      <c r="H98" s="2" t="inlineStr">
         <is>
           <t>Accepted</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H97"/>
+  <autoFilter ref="A1:H98"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
docs: record DEC-099 for the local workflow with checkpoints
Since #12 features and defects ran unattended in cloud sessions. STF-01
(#28) showed the cost: the owner saw only the result and interrupted
twice, four Needs decision items waited for a draft round, and the
sandbox got in the way (docker build without network, the proxy
footer, a read-only specification, no cache between sessions).

DEC-099: /implement-feature and /fix-defect run in Claude Code on the
owner's machine and stop at three checkpoints: the plan, where the
Needs decision items are asked; the failing tests; the diff before the
commit. Cloud sessions stay unattended for the routines and while the
owner is away. Reports and the metrics in issue #24 gain where and
owner-minutes; a pilot of three features decides whether it stays.

Refs: DEC-099
</commit_message>
<xml_diff>
--- a/docs/product-domain-blueprint-MVP.xlsx
+++ b/docs/product-domain-blueprint-MVP.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Workspaces\taitt0600\repos\zengear\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8F9257FD-B61F-4BB2-85FE-2D5AE2671E22}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{09B36E4E-860D-413C-BC5A-9FB85EB7E1F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="14180" windowWidth="25600" windowHeight="13900" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6380" uniqueCount="3410">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6388" uniqueCount="3416">
   <si>
     <t>Actor ID</t>
   </si>
@@ -11369,6 +11369,24 @@
   </si>
   <si>
     <t>DEC-098</t>
+  </si>
+  <si>
+    <t>DEC-099</t>
+  </si>
+  <si>
+    <t>Làm tính năng ở máy local có điểm duyệt</t>
+  </si>
+  <si>
+    <t>Từ PR #12, /implement-feature và /fix-defect chạy không người giám sát trong cloud session (CLAUDE.md, Workflow; DEC-098). Ở STF-01 (PR #28): chủ dự án chỉ thấy kết quả cuối và phải ngắt giữa chừng 2 lần (tên nhánh, footer); 4 mục Needs decision chỉ được hỏi sau khi PR mở, trả lời theo đề xuất nhưng vẫn tốn một vòng draft rồi ready; sandbox cloud: docker build không ra mạng (phải build bằng bản Dockerfile thêm proxy và CA), Docker daemon có lúc không trả lời, không có GraphQL, proxy tự gắn footer Generated by Claude Code vào PR và comment; spec và tooling chỉ đọc nên mọi thay đổi owner path phải soạn thành prompt dán sang phiên local; mỗi phiên không giữ cache (image acceptance build lại khoảng 25 phút). Đã so sánh: giữ cloud không người giám sát; làm ở local không điểm duyệt; làm ở local có điểm duyệt.</t>
+  </si>
+  <si>
+    <t>/implement-feature và /fix-defect chạy mặc định trong Claude Code trên máy chủ dự án (VS Code, hoặc Desktop chế độ Local), mỗi tính năng một nhánh feat/&lt;id&gt; hoặc fix/&lt;id&gt;-&lt;tên&gt; và một phiên; khi CLAUDE_CODE_REMOTE khác true, /implement-feature dừng đúng 3 điểm duyệt: (1) sau khi plan-reviewer trả READY, trình plan và hỏi ngay mọi mục Needs decision kèm phương án và đề xuất, câu trả lời thành quyết định đã chọn, câu trả lời làm đổi spec thì dừng và soạn Decision bằng /decision-draft; (2) sau khi viết test và thấy test đỏ, trình danh sách test theo rule ID; (3) trước khi commit, trình git diff --stat, kết quả build, test, review, acceptance và hỏi số phút chủ dự án đã tham gia; ngoài 3 điểm này Claude tự chạy theo chính sách quyết định của /implement-feature bước 4; /fix-defect dừng ở test tái hiện lỗi và trước khi commit. Cloud session vẫn chạy không người giám sát cho routine ZenGear fix defects và khi chủ dự án vắng; ở cloud, ngay sau khi mở PR, chuyển PR sang ready hoặc đăng comment, gỡ footer proxy gắn vào. Báo cáo nghiệm thu ghi hai dòng Nơi chạy (local hoặc cloud) và Thời gian bạn tham gia (phút, 0 ở cloud); routine ZenGear PR merged chép hai trường này vào dòng log ở issue #24. Thử 3 tính năng ở local bắt đầu từ STF-03, so với STF-01 và AUT-04 chạy ở cloud: giữ cách làm này khi lead time không tệ hơn 20%, số lỗi nghiệm thu không tăng và thời gian chủ dự án tham gia không quá 20 phút mỗi tính năng; không đạt thì quay về tính năng ở cloud, spec và tooling ở local. Mở rộng DEC-098: mọi bước vẫn dùng skill và script trong repo, chạy giống nhau ở cloud và local. Không chọn: giữ cloud không người giám sát (không lái được giữa chừng, quyết định dồn về cuối, ma sát sandbox); làm ở local không điểm duyệt (mất phần kiểm soát chủ dự án cần); duyệt từng thao tác (mệt vì duyệt quyền, dễ duyệt cho qua).</t>
+  </si>
+  <si>
+    <t>CLAUDE.md (Workflow), .claude/commands/implement-feature.md, finish-feature.md, fix-defect.md và docs/AUTOMATION.md đổi trong một pull request owner path do chủ dự án mở và merge; prompt của hai routine ZenGear PR merged và ZenGear PR needs decision cập nhật theo docs/AUTOMATION.md; máy phải bật trong lúc chạy và guard-spec hỏi xác nhận thay vì từ chối; ở local, PR mở bằng token gh của chủ dự án nên gate mở từ Claude app của tools/pr_gates.py không nhận ra, an toàn dựa vào xác nhận của guard, các luật deny (push main, --no-verify, gh pr merge), việc tools/github_pr.py từ chối auto-merge PR owner path và việc Claude không tự mở PR owner path; schema check vẫn bỏ qua ở local, CI chạy thay; khác biệt Windows và CI (python thay python3, file bị Visual Studio khóa, port emulator 9099 và 4000 dùng chung với môi trường acceptance) xử lý theo env_doctor; lý do không chọn LSP plugin trong DEC-098 (local không viết tính năng) không còn đúng, xem lại riêng khi cần; thời gian chủ dự án tham gia tăng nhưng có trần.</t>
+  </si>
+  <si>
+    <t>Chủ dự án; số liệu STF-01 (PR #28) trong cloud session ngày 2026-10-02; Claude Code docs: VS Code extension, Permission modes, Checkpointing</t>
   </si>
 </sst>
 </file>
@@ -29489,7 +29507,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
-  <dimension ref="A1:H99"/>
+  <dimension ref="A1:H100"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="11" customWidth="1"/>
@@ -32073,6 +32091,32 @@
         <v>15</v>
       </c>
       <c r="H99" s="2" t="s">
+        <v>2882</v>
+      </c>
+    </row>
+    <row r="100" spans="1:8" ht="178.5" x14ac:dyDescent="0.25">
+      <c r="A100" s="3" t="s">
+        <v>3410</v>
+      </c>
+      <c r="B100" s="2" t="s">
+        <v>3411</v>
+      </c>
+      <c r="C100" s="2" t="s">
+        <v>3412</v>
+      </c>
+      <c r="D100" s="2" t="s">
+        <v>3413</v>
+      </c>
+      <c r="E100" s="2" t="s">
+        <v>3414</v>
+      </c>
+      <c r="F100" s="2" t="s">
+        <v>3415</v>
+      </c>
+      <c r="G100" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="H100" s="2" t="s">
         <v>2882</v>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: record DEC-101 for the CI jobs, checks and Postman rules
Applying DEC-100 (#30, #31, #32) settled points its text left open or
put otherwise: package and acceptance became one job, so the image
tested is the image pushed; every job is named after its id in lower
case; the required checks are ci-ok, pr-gates and pr-title, pinned to
GitHub Actions; the collection needs fixed role ids, dev-only fixtures
and sign-in through emulator custom tokens; and in a private
repository required reviewers need GitHub Enterprise, so the approval
of a production deploy is decided when deploy is enabled.

DEC-101 records these rules and replaces the parts of DEC-100 (8) on
the package job, the names of the required checks and the approval by
environment. The Tech Stack rows of GitHub Actions and Postman follow.

Refs: DEC-101, DEC-100
</commit_message>
<xml_diff>
--- a/docs/product-domain-blueprint-MVP.xlsx
+++ b/docs/product-domain-blueprint-MVP.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Workspaces\taitt0600\repos\zengear\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EEDFE82F-7AD5-46E8-B28E-36BF1122B77D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1DD62584-03B3-4CB6-AD32-49D14DFAD10E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="14180" windowWidth="25600" windowHeight="13900" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6406" uniqueCount="3428">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6414" uniqueCount="3434">
   <si>
     <t>Actor ID</t>
   </si>
@@ -11416,13 +11416,31 @@
     <t>DEC-088, DEC-100, zengear_00_schema_full.sql</t>
   </si>
   <si>
-    <t>Một pipeline (pipeline.yml): job changes chọn job theo path; secrets, tools-test, api-test, schema, package (image và migration bundle build một lần), acceptance (collection Postman trên image đó), web-test và web-preview khi có web, ci-ok; gates.yml cho PR gates và tiêu đề PR; push main deploy staging, production sau khi duyệt (DEC-093, DEC-100)</t>
-  </si>
-  <si>
     <t>v12</t>
   </si>
   <si>
-    <t>Collection v3 lưu bằng Git gốc trong postman/, mỗi tính năng một folder; chủ dự án test trước khi merge; Postman CLI chạy collection trong CI và trên API dev (DEC-100)</t>
+    <t>DEC-101</t>
+  </si>
+  <si>
+    <t>Chốt CI/CD và Postman sau triển khai DEC-100</t>
+  </si>
+  <si>
+    <t>Ba pull request áp dụng DEC-100 (#30 công cụ, #31 Postman và workflow, #32 pipeline) cho thấy vài điểm văn bản DEC-100 ghi khác hoặc chưa nói: (a) DEC-100 (8) tách package và acceptance thành hai job, nhưng chuyển image giữa hai job tốn thời gian và image được kiểm thử có thể khác image được đẩy lên GHCR; (b) tên check lẫn chữ hoa và chữ thường (Scan for secrets, PR gates, Validate PR title, build-test) trong khi id job là chữ thường, và required checks khai bằng tên thì nhận kết quả từ mọi nguồn (any source); (c) gates.yml chạy bằng pull_request_target, tức bản trên main, nên đổi tên một job của nó phải đổi required checks hai lần quanh lúc merge; (d) repo private: environment và giới hạn nhánh cần GitHub Pro, required reviewers cần GitHub Enterprise, nên bước duyệt production bằng environment như DEC-100 (8) có thể không dùng được; (e) collection Postman cần ID role cố định (chưa có endpoint liệt kê role), một trạng thái API chưa tạo được (người không phải Admin giữ staff.create và không phải đổi mật khẩu, cho R-TX-11) và cách đăng nhập không mật khẩu, còn Postman app ghi biến collection ngược vào file. Đo ngày 2026-10-02 trên PR #32: thời gian CI trung vị 3 lần chạy 3 phút 22 giây (lần cache trống 6 phút 16 giây, hai lần sau chạy lại cùng commit); trong job acceptance, bước chậm nhất là migration bundle 50 đến 66 giây.</t>
+  </si>
+  <si>
+    <t>(1) Tên job trong .github/workflows trùng id job, chữ thường nối bằng gạch: pipeline.yml gồm changes, secrets, tools-test, api-test, schema, acceptance, ci-ok, deploy-staging, deploy-production; gates.yml (pull_request_target) gồm pr-gates, pr-title; tools/tests/test_github_pr.py kiểm quy tắc này. (2) Required checks của main là ci-ok, pr-gates, pr-title, mỗi check gắn nguồn GitHub Actions (app_id 15368), giữ Require branches to be up to date và Do not allow bypassing; REQUIRED_CHECKS của tools/github_pr.py trùng danh sách này; đổi tên một job của gates.yml thì đổi required checks hai lần: tên cũ trước khi merge, tên mới ngay sau khi merge. (3) package gộp vào job acceptance: build image API (buildx, cache gha) và migration bundle một lần, dựng compose của CI từ đúng image đó, chuẩn bị dữ liệu trước khi API khởi động theo thứ tự của tools/dev_reset.ps1 (init, Admin bằng bootstrap-admin, fixture), chạy toàn bộ collection, trên main đẩy chính image đó lên GHCR và lưu bundle cho deploy; output của bootstrap-admin không bao giờ vào log. (4) Concurrency: mỗi pull request chỉ giữ run mới nhất; mỗi run trên main có group riêng theo SHA, không hủy và không thay nhau; deploy-staging và deploy-production mỗi job một group, chạy lần lượt. (5) Postman: 9 role của api/seed/01_roles.sql mang ID cố định, không bao giờ đổi; trạng thái API chưa tạo được dựng bằng fixture chỉ dùng cho dev và CI trong postman/fixtures (tài khoản emulator theo accounts.txt, SQL chạy sau seed và trước khi API khởi động), không bao giờ vào seed, staging hay production, và bỏ khi API tạo được trạng thái đó (fixture của STF-01 bỏ khi có STF-03 và AUT-05); collection đăng nhập bằng custom token không ký của Firebase Auth Emulator qua header X-ZenGear-As, chỉ chạy với emulator trên localhost; script giữ trạng thái của lần chạy trong pm.variables, không dùng biến collection, environment hay globals; .postman/ và postman/globals/ không commit; Postman CLI 1.69.0 cài bằng npm. (6) Cơ chế duyệt deploy production (environment có required reviewers, cần GitHub Enterprise với repo private, hoặc workflow_dispatch chạy tay) và smoke test đăng nhập thật trên staging quyết định khi bật deploy. Thay thế phần của DEC-100 (8) về job package riêng, tên required checks (PR gates, Validate PR title) và bước duyệt production bằng environment. Không chọn: package và acceptance là hai job (chuyển image khoảng 365 MB qua artifact, image kiểm thử có thể khác image đẩy); giữ tên check cũ (lẫn kiểu chữ, khác id job); required checks any source (một commit status cùng tên gửi bằng token cá nhân cũng được tính); lấy ID role qua endpoint (chưa có endpoint); tạo trạng thái của R-TX-11 qua API (cần STF-03 và AUT-05); mật khẩu test trong collection (secret trong repo); bỏ qua request cần fixture trong CI (mất phép kiểm R-TX-11).</t>
+  </si>
+  <si>
+    <t>Spec khớp với pipeline.yml, gates.yml và tools/github_pr.py đã merge ở #32, và với postman/, api/seed/01_roles.sql, tools/dev_reset.ps1 đã merge ở #31; không đổi code. Đổi tên một job bắt buộc của gates.yml luôn cần hai lần đổi required checks; job mới trong pipeline chỉ cần thêm vào needs của ci-ok. Người duyệt pull request sửa .github/ phải kiểm không có job nào khác tên ci-ok, pr-gates hay pr-title: gắn nguồn GitHub Actions không chặn được một job trùng tên. Fixture phải giữ khớp giữa tools/dev_reset.ps1 và job acceptance; mỗi fixture hết hạn khi tính năng tạo được trạng thái đó. Thời gian CI thật đo ở pull request tính năng đầu tiên có sửa api/ (dự kiến thêm khoảng 1 phút vì build lại image); vượt 3 phút 30 giây thì áp dụng một trong hai: build bundle chạy nền song song với build image, hoặc NuGet cache bằng actions/cache. Cần quyết định khi bật deploy: mục (6), cộng các mục đã nêu ở DEC-100.</t>
+  </si>
+  <si>
+    <t>Chủ dự án; PR #30, #31, #32; số liệu CI của PR #32 ngày 2026-10-02; GitHub docs: Managing environments for deployment, Deployments and environments, About protected branches (required status checks), Control the concurrency of workflows and jobs; Postman docs: Variables (scopes), Postman CLI; Firebase docs: Connect your app to the Authentication Emulator</t>
+  </si>
+  <si>
+    <t>Một pipeline (pipeline.yml), tên job trùng id: changes chọn job theo path; secrets, tools-test, api-test, schema, acceptance (build image và migration bundle một lần, chạy toàn bộ collection Postman trên image đó, trên main đẩy image lên GHCR), web-test và web-preview khi có web, ci-ok; gates.yml: pr-gates, pr-title; required checks ci-ok, pr-gates, pr-title; push main deploy staging rồi production (DEC-093, DEC-100, DEC-101)</t>
+  </si>
+  <si>
+    <t>Collection v3 lưu bằng Git gốc trong postman/, mỗi tính năng một folder; chủ dự án test trước khi merge; Postman CLI 1.69.0 chạy collection trong CI và trên API dev, không cần đăng nhập; collection đăng nhập bằng custom token của Firebase Auth Emulator (DEC-100, DEC-101)</t>
   </si>
 </sst>
 </file>
@@ -11478,7 +11496,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -11490,9 +11508,6 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -12933,7 +12948,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="40" spans="1:5" ht="38.25" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:5" ht="51" x14ac:dyDescent="0.25">
       <c r="A40" s="2" t="s">
         <v>178</v>
       </c>
@@ -12941,10 +12956,10 @@
         <v>183</v>
       </c>
       <c r="C40" s="2" t="s">
-        <v>3426</v>
+        <v>3425</v>
       </c>
       <c r="D40" s="2" t="s">
-        <v>3427</v>
+        <v>3433</v>
       </c>
       <c r="E40" s="2" t="s">
         <v>15</v>
@@ -13018,7 +13033,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="45" spans="1:5" ht="76.5" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:5" ht="89.25" x14ac:dyDescent="0.25">
       <c r="A45" s="2" t="s">
         <v>189</v>
       </c>
@@ -13029,7 +13044,7 @@
         <v>74</v>
       </c>
       <c r="D45" s="2" t="s">
-        <v>3425</v>
+        <v>3432</v>
       </c>
       <c r="E45" s="2" t="s">
         <v>15</v>
@@ -29588,7 +29603,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
-  <dimension ref="A1:H101"/>
+  <dimension ref="A1:H102"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="11" customWidth="1"/>
@@ -32175,7 +32190,7 @@
         <v>3422</v>
       </c>
     </row>
-    <row r="100" spans="1:8" ht="357" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:8" ht="178.5" x14ac:dyDescent="0.25">
       <c r="A100" s="3" t="s">
         <v>3406</v>
       </c>
@@ -32201,8 +32216,8 @@
         <v>3422</v>
       </c>
     </row>
-    <row r="101" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
-      <c r="A101" s="5" t="s">
+    <row r="101" spans="1:8" ht="178.5" x14ac:dyDescent="0.25">
+      <c r="A101" s="3" t="s">
         <v>3412</v>
       </c>
       <c r="B101" s="2" t="s">
@@ -32224,6 +32239,32 @@
         <v>15</v>
       </c>
       <c r="H101" s="2" t="s">
+        <v>2880</v>
+      </c>
+    </row>
+    <row r="102" spans="1:8" ht="178.5" x14ac:dyDescent="0.25">
+      <c r="A102" s="3" t="s">
+        <v>3426</v>
+      </c>
+      <c r="B102" s="2" t="s">
+        <v>3427</v>
+      </c>
+      <c r="C102" s="2" t="s">
+        <v>3428</v>
+      </c>
+      <c r="D102" s="2" t="s">
+        <v>3429</v>
+      </c>
+      <c r="E102" s="2" t="s">
+        <v>3430</v>
+      </c>
+      <c r="F102" s="2" t="s">
+        <v>3431</v>
+      </c>
+      <c r="G102" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="H102" s="2" t="s">
         <v>2880</v>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: record DEC-107 for the rollout of DEC-106
DEC-107 amends DEC-106 with what its rollout (#51 to #54) changed:
[ShopEndpoint] holds only the anonymous access, and the rate limit
and output cache of the shop wait for their own Decision; an admin
list of business locations keeps the 405 of R-LOC-01; two controllers
keep their resource names; the route break stays in v1; the paging
rule is not shared yet; the access-surface tests live in the
integration tests; a feature creates the modules of a listed area;
Claude writes PRD-02 and issue #24 logs the labelled findings and the
folders per feat commit.

Refs: DEC-107, DEC-106, LOC-01
</commit_message>
<xml_diff>
--- a/docs/product-domain-blueprint-MVP.xlsx
+++ b/docs/product-domain-blueprint-MVP.xlsx
@@ -24,7 +24,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Use Cases'!$A$1:$L$140</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Domain Model'!$A$1:$J$78</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Business Rules'!$A$1:$I$137</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Decisions'!$A$1:$H$107</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Decisions'!$A$1:$H$108</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Technical Design'!$A$1:$E$17</definedName>
   </definedNames>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -30832,7 +30832,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H107"/>
+  <dimension ref="A1:H108"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -35339,8 +35339,50 @@
         </is>
       </c>
     </row>
+    <row r="108" ht="409.5" customHeight="1">
+      <c r="A108" s="3" t="inlineStr">
+        <is>
+          <t>DEC-107</t>
+        </is>
+      </c>
+      <c r="B108" s="2" t="inlineStr">
+        <is>
+          <t>Điều chỉnh DEC-106 sau khi triển khai</t>
+        </is>
+      </c>
+      <c r="C108" s="2" t="inlineStr">
+        <is>
+          <t>DEC-106 được triển khai qua PR #51 (docs/CODING_GUIDE.md), #52 (cấu trúc Area/Module), #53 và #54 (route admin và shop); trong lúc làm có chín điểm không làm đúng chữ được: (a) code chưa có rate limit hay output cache nào, con số giới hạn cần traffic thật, và danh sách địa điểm kinh doanh có giờ mở cửa tính từ hôm nay theo Asia/Ho_Chi_Minh nên cache qua nửa đêm sẽ hiện giờ của ngày hôm trước; (b) danh sách địa điểm của shop và GET, PUT theo id của admin dùng chung route api/v1/business-locations, tách ra thì POST lên collection admin trả 404 thay 405 (test R-LOC-01, Postman LOC-01/05, docs/API_CONVENTIONS.md) và màn SCR-LOC-01 phải gọi API shop để lấy id; (c) đổi tên MeController và BusinessLocationsController theo tên service làm đổi tag OpenAPI thêm một lần; (d) docs/API_CONVENTIONS.md bắt breaking change lên version mới, nhưng client duy nhất là collection Postman và test; (e) StaffListRequestValidator trả lỗi phân trang kèm ruleId R-USR-13 và message riêng (test STF-05, Postman STF-05/13), còn validator PageRequest của Common không có mã rule, dùng chung bằng Include sẽ mất ruleId; (f) kiểm route và quyền ẩn danh cần tập endpoint sau khi convention chạy, ZenGear.ArchitectureTests không có package dựng host và thêm package cần Decision; (g) [ShopEndpoint] là IAllowAnonymous cấp class nên thắng mọi quyền khai báo trên action; (h) chủ dự án chỉ tự code khi không có mạng hoặc không truy cập được Claude, nên đo bằng cách tự viết PRD-02 không còn hợp; (i) bước 4 của /implement-feature coi mọi folder mới là Needs decision, với cấu trúc module thì tính năng đầu của mỗi area đều dừng lại hỏi. Đã so sánh từng điểm: làm đúng chữ DEC-106, hoãn, hoặc điều chỉnh như dưới.</t>
+        </is>
+      </c>
+      <c r="D108" s="2" t="inlineStr">
+        <is>
+          <t>Sửa DEC-106 như sau, phần còn lại giữ nguyên. (1) [ShopEndpoint] (sealed, cấp class, IAllowAnonymous) chỉ cho truy cập ẩn danh và đánh dấu endpoint shop; rate limit và output cache của shop đi cùng một Decision riêng trước khi deploy storefront, trong đó cache danh sách địa điểm phải hết hạn trước nửa đêm giờ Asia/Ho_Chi_Minh; endpoint shop cần khách đăng nhập (AUT-02, MeShopController) và callback thanh toán (VNPay IPN) cần một Decision sửa [ShopEndpoint] và test của nó trước khi viết. (2) Thêm GET /api/v1/admin/business-locations: nhận PageRequest, trả PagedDto&lt;BusinessLocationDto&gt;, quyền business_location.update (seed không đổi), sắp theo name rồi id; SCR-LOC-01 lấy id địa điểm từ đây; POST lên collection admin vẫn trả 405 (R-LOC-01). (3) MeController và BusinessLocationsController giữ tên theo resource; đổi tên sau này phải chấp nhận đổi tag OpenAPI. (4) Việc chuyển route sang hai prefix giữ ở v1 vì client duy nhất là collection Postman và test; từ nay breaking change lên version mới như docs/API_CONVENTIONS.md. (5) Quy tắc phân trang chưa dùng chung: mỗi rule giữ mã lỗi riêng (lặp có chủ ý, docs/CODING_GUIDE.md mục 3); dùng chung cần một rule-builder trong Common nhận mã của nơi gọi, loại type mới mà docs/ARCHITECTURE.md bắt hỏi trước. (6) Kiểm tra bề mặt truy cập là test của ZenGear.Api.IntegrationTests (Authorization/AccessSurfaceTests) đọc EndpointDataSource: mọi route dưới /api/v1/admin/ hoặc /api/v1/shop/; endpoint ẩn danh khi và chỉ khi nằm dưới shop và qua [ShopEndpoint]; endpoint shop không mang quyền hay [AnyRegisteredUser]; action shop chỉ trả *ShopDto hoặc PagedDto&lt;*ShopDto&gt;; mỗi kiểm tra có mẫu tự chứng minh nó báo lỗi được; convention AudienceRoutePrefixConvention (ZenGear.Api/Hosting) ném lỗi khi dựng application model nếu controller thiếu [Route], route bắt đầu bằng api/, / hoặc ~/, hay action có route tuyệt đối, nên build sinh OpenAPI và test đều đỏ. (7) Folder mới: tính năng tự tạo module của một area đã có trong bảng của docs/ARCHITECTURE.md (kèm dòng dưới Modules trong README của area, và README khi tạo module đầu) cùng các folder Controllers, Entities, Configurations và test của area đó, ghi vào mục Decisions made của báo cáo; area mới, folder cơ chế, folder kỹ thuật của ZenGear.Api hay ZenGear.Data, folder trong Common vẫn là Needs decision. (8) Đo: Claude viết PRD-02 và các tính năng sau theo DEC-106 và docs/CODING_GUIDE.md; báo cáo nghiệm thu có dòng Phát hiện over-engineering / duplication và Folder mỗi commit feat (tools/structure_metrics.py --range), ghi ? khi lần chạy dừng trước code review; routine ZenGear PR merged và ZenGear PR needs decision chép vào issue #24 thành over-engineering, duplication và folders per feat commit; riêng PRD-02 chủ dự án ghi thêm có tìm thấy code trong không quá 3 folder không; phép đo khi tự code của DEC-106 (thời gian, số lần tra tài liệu hay hỏi Claude, số vòng CI đỏ) làm vào lần tới chủ dự án tự code. Không chọn: thêm rate limit và output cache ngay (chưa có traffic để chọn con số, dễ cache sai ngày); chấp nhận 404 cho POST và để màn admin đọc danh sách shop (nới test R-LOC-01, trộn hai phía DEC-106 muốn tách); đổi tên hai controller ngay (đổi tag OpenAPI thêm một lần mà không được gì); lên v2 (không client nào cần giữ v1); dùng chung quy tắc phân trang bằng Include validator (mất ruleId R-USR-13, phá test STF-05); thêm package dựng host vào ZenGear.ArchitectureTests (cần Decision, test tích hợp đã có host); giữ mọi folder mới là Needs decision (tính năng đầu của mỗi area đều dừng hỏi); chủ dự án tự viết PRD-02 (chỉ tự code khi không có Claude).</t>
+        </is>
+      </c>
+      <c r="E108" s="2" t="inlineStr">
+        <is>
+          <t>Các điểm trên đã có trong code và tài liệu từ PR #51 đến #54: docs/CODING_GUIDE.md (Status), docs/API_CONVENTIONS.md (URLs, Authentication), docs/ARCHITECTURE.md (Folder structure), api/CLAUDE.md, docs/SCREENS.md (SCR-LOC-01), .claude/commands/implement-feature.md (bước 4) và finish-feature.md (bước 14), agent report-reviewer, skill report-review, docs/AUTOMATION.md; pull request ghi DEC-107 chỉ đổi workbook và docs/blueprint/, sau đó một pull request tài liệu đổi các câu "một /decision-draft sau sẽ sửa DEC-106" trong docs/CODING_GUIDE.md và docs/API_CONVENTIONS.md thành DEC-107; prompt hai routine ZenGear PR merged và ZenGear PR needs decision đã cập nhật ngày 2026-10-10; API có 12 endpoint (thêm danh sách admin), 486 test, collection Postman 91 request; FallbackPolicy đã có từ trước nên refactor B không phải thêm; comment trong api/src giảm từ 986 xuống 937 dòng; trước khi bật deploy storefront phải có Decision về rate limit và output cache của shop, trước khi viết AUT-02 phải có Decision sửa [ShopEndpoint]; bảng ngưỡng tiến hóa và cấu trúc của DEC-106 không đổi.</t>
+        </is>
+      </c>
+      <c r="F108" s="2" t="inlineStr">
+        <is>
+          <t>Chủ dự án (quyết định D1, D2 và các câu trả lời ngày 2026-10-10); DEC-106; DEC-105; PR #51, #52, #53, #54; issue #24; ASP.NET Core (IControllerModelConvention, IAllowAnonymous, EndpointDataSource)</t>
+        </is>
+      </c>
+      <c r="G108" s="2" t="inlineStr">
+        <is>
+          <t>Phase 1</t>
+        </is>
+      </c>
+      <c r="H108" s="2" t="inlineStr">
+        <is>
+          <t>Accepted</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:H107"/>
+  <autoFilter ref="A1:H108"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
docs: record DEC-108 for moving R-PRD-07 to PRD-05
Refs: DEC-108, PRD-02, PRD-03, PRD-05, R-PRD-07
</commit_message>
<xml_diff>
--- a/docs/product-domain-blueprint-MVP.xlsx
+++ b/docs/product-domain-blueprint-MVP.xlsx
@@ -24,7 +24,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Use Cases'!$A$1:$L$140</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Domain Model'!$A$1:$J$78</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Business Rules'!$A$1:$I$137</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Decisions'!$A$1:$H$108</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Decisions'!$A$1:$H$109</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Technical Design'!$A$1:$E$17</definedName>
   </definedNames>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -3688,13 +3688,12 @@
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>- Brand là entity độc lập, không nằm trong JSONB attributes.
-- Mỗi Product bắt buộc gán 1 Brand.</t>
+          <t>- Brand là entity độc lập, không nằm trong JSONB attributes.</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>R-PRD-07, R-DEL-01</t>
+          <t>R-DEL-01</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
@@ -3746,13 +3745,12 @@
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>- 1 Series luôn thuộc đúng 1 Brand.
-- 1 Product thuộc tối đa 1 Series (nullable).</t>
+          <t>- 1 Series luôn thuộc đúng 1 Brand.</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>R-PRD-07, R-DEL-01</t>
+          <t>R-DEL-01</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
@@ -3865,12 +3863,13 @@
           <t>- SKU duy nhất, không đổi sau khi tạo; attributes validate theo attribute_schema.
 - Sản phẩm bảo hành theo Serial (CPU/GPU/Mainboard) khai báo requires_serial=true; requires_serial chỉ đổi được khi chưa từng có tồn kho và chưa từng bán (R-PRD-08).
 - Bắt buộc gán tax_class_id (nhóm tính thuế GTGT theo % doanh thu, TAX-01); mọi SKU của sản phẩm dùng chung nhóm.
-- Lưu dùng optimistic concurrency (xmin): người lưu sau được báo tải lại, không ghi đè (R-TX-15).</t>
+- Lưu dùng optimistic concurrency (xmin): người lưu sau được báo tải lại, không ghi đè (R-TX-15).
+- Mỗi Product gán đúng 1 Brand và tối đa 1 Series; có Series thì Brand của Series phải trùng Brand của Product (R-PRD-07).</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>R-PRD-01, R-PRD-03, R-PRD-05, R-PRD-08, R-TX-15</t>
+          <t>R-PRD-01, R-PRD-03, R-PRD-05, R-PRD-07, R-PRD-08, R-TX-15</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
@@ -25495,7 +25494,7 @@
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>PRD-02, PRD-03</t>
+          <t>PRD-05</t>
         </is>
       </c>
       <c r="H24" s="2" t="inlineStr">
@@ -30832,7 +30831,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H108"/>
+  <dimension ref="A1:H109"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -35381,8 +35380,50 @@
         </is>
       </c>
     </row>
+    <row r="109" ht="409.5" customHeight="1">
+      <c r="A109" s="3" t="inlineStr">
+        <is>
+          <t>DEC-108</t>
+        </is>
+      </c>
+      <c r="B109" s="2" t="inlineStr">
+        <is>
+          <t>R-PRD-07 chuyển sang tính năng tạo Product</t>
+        </is>
+      </c>
+      <c r="C109" s="2" t="inlineStr">
+        <is>
+          <t>R-PRD-07 (có Series thì Brand của Series phải trùng Brand của Product; mỗi Product đúng 1 Brand, tối đa 1 Series) ghi Enforced At là Service — Product aggregate trên products, product_series, brands, nhưng cột Features chỉ có PRD-02 (Manage Brand) và PRD-03 (Manage Product Series); tính năng tạo bảng products và Product aggregate là PRD-05 lại không ghi rule này. PRD-02 chỉ tạo bảng brands, PRD-03 chỉ tạo product_series, nên không tính năng nào trong hai cái dựng hay kiểm thử được rule; tiêu chí 'Mỗi Product bắt buộc gán 1 Brand' của PRD-02 và '1 Product thuộc tối đa 1 Series (nullable)' của PRD-03 cũng là về Product. PR-gates đòi mỗi rule của tính năng có test tên R_PRD_07_…, nên PR của PRD-02 (feat/prd-02, chủ dự án chọn làm trước, để PR draft) chỉ còn trượt ở R-PRD-07; một test đặt tên R-PRD-07 ở PRD-02 chỉ qua cổng mà không chứng minh rule. Khi products được migrate, products.brand_id NOT NULL và FK ghép fk_products_product_series_series_id (series_id, brand_id) → product_series (id, brand_id) giữ rule ở database, Product aggregate kiểm trước để báo lỗi rõ. Phương án đã so sánh: chuyển rule và hai tiêu chí sang PRD-05; giữ ở PRD-03 phần Series; đưa bảng products, product_series, categories, tax_classes lên làm sớm trong PRD-02.</t>
+        </is>
+      </c>
+      <c r="D109" s="2" t="inlineStr">
+        <is>
+          <t>R-PRD-07 thuộc PRD-05: cột Features của R-PRD-07 chỉ còn PRD-05; PRD-02 và PRD-03 bỏ R-PRD-07 khỏi cột Rules và bỏ tiêu chí về Product ('Mỗi Product bắt buộc gán 1 Brand', '1 Product thuộc tối đa 1 Series (nullable)'); PRD-05 thêm R-PRD-07 vào Rules và một tiêu chí: mỗi Product gán đúng 1 Brand và tối đa 1 Series, có Series thì Brand của Series phải trùng Brand của Product. Test R_PRD_07_… viết ở PRD-05: Product aggregate từ chối Product thiếu Brand hoặc Series khác Brand, và database từ chối qua NOT NULL và FK ghép. PRD-02 giữ R-DEL-01 và tiêu chí Brand là entity độc lập; PRD-03 giữ R-DEL-01 và tiêu chí 1 Series thuộc đúng 1 Brand. Không chọn: giữ R-PRD-07 ở PRD-03 cho phần Series, vì product_series một mình không thể hiện được rule và PRD-03 sẽ vướng cùng cổng PR-gates; làm sớm products và các bảng nó cần trong PRD-02, vì vượt xa phạm vi Manage Brand và kéo theo nhóm thuế, danh mục.</t>
+        </is>
+      </c>
+      <c r="E109" s="2" t="inlineStr">
+        <is>
+          <t>PR PRD-02 qua PR-gates sau khi rebase lên main có DEC-108 (cổng đọc Rules ở cả base và head); PRD-03 làm được mà không cần Decision riêng cho R-PRD-07; PRD-05 có thêm một rule và một tiêu chí phải có test và kịch bản Postman. Không đổi schema, docs/DATABASE.md hay api/db. Cột Depends On đang ghi tên Epic nên không thêm PRD-02, PRD-03 vào PRD-05; khi làm PRD-05 cần sẵn bảng brands (PRD-02) và product_series (PRD-03). Domain Model vẫn ghi R-PRD-07 ở Brand và Product: đó là bất biến của aggregate, không phải tính năng nào kiểm thử.</t>
+        </is>
+      </c>
+      <c r="F109" s="2" t="inlineStr">
+        <is>
+          <t>Chủ dự án (PRD-02, 2026-10-14)</t>
+        </is>
+      </c>
+      <c r="G109" s="2" t="inlineStr">
+        <is>
+          <t>Phase 1</t>
+        </is>
+      </c>
+      <c r="H109" s="2" t="inlineStr">
+        <is>
+          <t>Accepted</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:H108"/>
+  <autoFilter ref="A1:H109"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
docs: record DEC-109 for a shared paging helper
DEC-109 adds PagedQuery at the root of ZenGear.Services/Common: one
ToPagedDtoAsync over an ordered query, a PageRequest and an optional
map, which skips the COUNT when the first page is not full. It
replaces the four copies of that code (staff, the two business
location lists, brands) before PRD-03 adds a fifth. Code shared by
the modules of one area gets no rule yet: CatalogSlug stays in
Catalog/Brands until a third module needs it.

Refs: DEC-109, DEC-106, DEC-107
</commit_message>
<xml_diff>
--- a/docs/product-domain-blueprint-MVP.xlsx
+++ b/docs/product-domain-blueprint-MVP.xlsx
@@ -24,7 +24,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Use Cases'!$A$1:$L$140</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Domain Model'!$A$1:$J$78</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Business Rules'!$A$1:$I$137</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Decisions'!$A$1:$H$109</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Decisions'!$A$1:$H$110</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Technical Design'!$A$1:$E$17</definedName>
   </definedNames>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -30831,7 +30831,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H109"/>
+  <dimension ref="A1:H110"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -35422,8 +35422,50 @@
         </is>
       </c>
     </row>
+    <row r="110" ht="409.5" customHeight="1">
+      <c r="A110" s="3" t="inlineStr">
+        <is>
+          <t>DEC-109</t>
+        </is>
+      </c>
+      <c r="B110" s="2" t="inlineStr">
+        <is>
+          <t>Helper phân trang dùng chung trong Common</t>
+        </is>
+      </c>
+      <c r="C110" s="2" t="inlineStr">
+        <is>
+          <t>Mỗi endpoint danh sách trả PagedDto&lt;T&gt; và bỏ câu COUNT khi trang đầu chưa đầy (trang đó đã chứa mọi dòng); đoạn code này được chép ở 4 service: StaffService (STF-05), BusinessLocationService và BusinessLocationShopService (LOC-01, DEC-107 (2)), BrandService (PRD-02); code-reviewer của PRD-02 gắn nhãn [duplication] và docs/CODING_GUIDE.md mục 3 bắt gom từ bản chép thứ ba; PRD-03 (danh sách Series) sẽ là bản thứ năm. Gom lại cần một type mới dùng EF Core (CountAsync, ToListAsync), nên không được xếp vào Common/Utilities (chỉ hàm thuần, không framework hay database), còn gốc ZenGear.Services/Common chỉ cho phép danh sách type ghi trong docs/ARCHITECTURE.md (IClock và Clock, BusinessRuleException, AdvisoryLockKeys), và hậu tố *Extensions chỉ dùng trong ZenGear.Api/Extensions. Câu hỏi đi kèm: code dùng chung giữa các module của một area (CatalogSlug, thuật toán slug của R-PRD-06, nằm trong Catalog/Brands mà Series, Category, Product sau này cũng cần) chưa có chỗ, vì gốc area chỉ chứa README và các module (DEC-106 (1)). Đã so sánh: static class PagedQuery ở gốc Common; factory tĩnh trên PagedDto; giữ các bản chép; với code dùng chung trong area: chưa đặt quy tắc hoặc thêm folder &lt;Area&gt;/Shared.</t>
+        </is>
+      </c>
+      <c r="D110" s="2" t="inlineStr">
+        <is>
+          <t>(1) Thêm static class PagedQuery ở gốc ZenGear.Services/Common với một hàm ToPagedDtoAsync nhận query đã lọc và sắp xếp (thứ tự ổn định do nơi gọi đặt, ví dụ theo name rồi id), PageRequest, CancellationToken và một hàm map từ dòng sang DTO (không truyền thì dòng chính là DTO); hàm lấy trang bằng Skip và Take, map trong bộ nhớ, và chỉ chạy COUNT trên cùng query khi không phải trang đầu hoặc trang đầu đã đầy; trả PagedDto&lt;T&gt;. Hàm không validate PageRequest: service vẫn gọi validator PageRequest (hay validator riêng của danh sách, như R-USR-13 của STF-05) trước. StaffService, BusinessLocationService, BusinessLocationShopService và BrandService dùng PagedQuery; mỗi endpoint danh sách sau này cũng vậy. docs/ARCHITECTURE.md thêm PagedQuery vào danh sách type của gốc Common. PagedQuery có unit test cho trang đầu chưa đầy (không COUNT), trang đầu đầy và trang sau (có COUNT), trang quá cuối (danh sách rỗng, totalCount đúng). (2) Chưa đặt quy tắc cho code dùng chung giữa các module của một area: CatalogSlug ở lại Catalog/Brands, module khác của Catalog gọi sang đó (cùng area được phép, quy tắc 4 chỉ giới hạn lời gọi giữa các area); khi module thứ ba cần một type như vậy thì mở Decision về chỗ đặt. Không chọn: factory tĩnh trên PagedDto (DTO mang logic truy vấn EF, trái quy tắc DTO chỉ mang dữ liệu và Mapping); giữ các bản chép (sửa một chỗ phải sửa nhiều nơi, mỗi danh sách mới thêm một bản); extension method trong class *Extensions (hậu tố đó chỉ thuộc ZenGear.Api/Extensions); thêm folder &lt;Area&gt;/Shared ngay (mới một module dùng, YAGNI, và phải sửa test kiến trúc).</t>
+        </is>
+      </c>
+      <c r="E110" s="2" t="inlineStr">
+        <is>
+          <t>Một pull request refactor không đổi hành vi: thêm PagedQuery và unit test, 4 service chuyển sang dùng nó, OpenAPI và mọi test tích hợp, Postman giữ nguyên; docs/ARCHITECTURE.md đổi nên đây là owner path, chủ dự án mở và merge; không đổi schema, docs/DATABASE.md hay api/db; làm trước PRD-03 để danh sách Series dùng ngay PagedQuery. DEC-107 (5) không đổi: quy tắc validate phân trang của danh sách nhân viên vẫn giữ mã R-USR-13 riêng. Khi Catalog có module thứ ba cần CatalogSlug hoặc một type dùng chung khác, mở Decision về chỗ đặt code dùng chung trong một area.</t>
+        </is>
+      </c>
+      <c r="F110" s="2" t="inlineStr">
+        <is>
+          <t>Chủ dự án (hai lựa chọn ngày 2026-10-14); DEC-106; DEC-107; docs/CODING_GUIDE.md mục 3; PR #57 (code-reviewer, phát hiện [duplication])</t>
+        </is>
+      </c>
+      <c r="G110" s="2" t="inlineStr">
+        <is>
+          <t>Phase 1</t>
+        </is>
+      </c>
+      <c r="H110" s="2" t="inlineStr">
+        <is>
+          <t>Accepted</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:H109"/>
+  <autoFilter ref="A1:H110"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
docs: record DEC-114 for the prefetch and 404 of the nonce csp
DEC-114 aligns DEC-113 with pull request #85: src/proxy.ts skips only
the router prefetches, so that a browser prefetch of a document gets
the CSP with a nonce, and an unknown URL under /admin or /pos keeps
the static 404 until a catch-all route comes with STF-03 and with the
first POS screen. No x-nonce header is set while nothing reads it.

docs/STATUS.md loses the row dec-113-prefetch.

Refs: DEC-114, DEC-113
</commit_message>
<xml_diff>
--- a/docs/product-domain-blueprint-MVP.xlsx
+++ b/docs/product-domain-blueprint-MVP.xlsx
@@ -24,7 +24,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Use Cases'!$A$1:$L$140</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Domain Model'!$A$1:$J$78</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Business Rules'!$A$1:$I$137</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Decisions'!$A$1:$H$114</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Decisions'!$A$1:$H$115</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Technical Design'!$A$1:$E$17</definedName>
   </definedNames>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -30198,7 +30198,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H114"/>
+  <dimension ref="A1:H115"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -34999,8 +34999,50 @@
         </is>
       </c>
     </row>
+    <row r="115" ht="409.5" customHeight="1">
+      <c r="A115" s="3" t="inlineStr">
+        <is>
+          <t>DEC-114</t>
+        </is>
+      </c>
+      <c r="B115" s="2" t="inlineStr">
+        <is>
+          <t>Prefetch và trang 404 của CSP có nonce</t>
+        </is>
+      </c>
+      <c r="C115" s="2" t="inlineStr">
+        <is>
+          <t>DEC-113 (1) cho proxy.ts bỏ qua request prefetch (header next-router-prefetch hoặc purpose: prefetch) như hướng dẫn CSP của Next.js, và DEC-113 (3) ghi không trang nào dưới /admin và /pos render tĩnh. Khi áp DEC-113 (PR #85, Next.js 16.4.2): /admin và /pos không còn nhận CSP tĩnh của next.config.ts, nên một request mà proxy bỏ qua không mang CSP nào; prefetch của router (next-router-prefetch) chỉ tải payload RSC, không bao giờ là tài liệu, và một lần điều hướng không mang header đó; còn prefetch tài liệu của trình duyệt (Purpose hoặc Sec-Purpose: prefetch) có thể được trình duyệt hiển thị như trang, tức một trang không có CSP. URL không khớp trang nào dưới /admin, và mọi URL /pos lúc này, nhận trang 404 gốc mà Next.js render sẵn lúc build: trang đó không có nonce nên script của nó bị chặn, chữ 404 vẫn hiện. Chủ dự án trả lời cả hai điểm trong lúc chạy PR #85. Đã so sánh: bỏ qua cả hai loại prefetch như tài liệu; chỉ bỏ qua prefetch của router; với trang 404: thêm route catch-all ngay, hoặc thêm cùng màn hình kế tiếp.</t>
+        </is>
+      </c>
+      <c r="D115" s="2" t="inlineStr">
+        <is>
+          <t>(1) Thay phần prefetch của DEC-113 (1): proxy.ts chỉ bỏ qua request có header next-router-prefetch; prefetch tài liệu của trình duyệt (Purpose hoặc Sec-Purpose: prefetch) nhận CSP có nonce như mọi lần tải; một điều kiện bỏ qua thêm sau này phải giữ CSP trên mọi response là tài liệu. (2) Làm rõ DEC-113 (3): route catch-all gọi notFound() nằm dưới layout của /admin (đến cùng PR web-only của STF-03) và dưới layout của /pos (đến cùng màn hình POS đầu tiên), để URL không tồn tại render 404 có nonce; cho tới đó URL không tồn tại dưới hai nhánh này nhận 404 tĩnh không có nonce, chấp nhận vì script bị chặn mà không lộ gì. (3) Không đặt header x-nonce khi chưa có code đọc nó; Script nào cần nonce đọc nó từ header content-security-policy của request (docs/FRONTEND.md). Không chọn: bỏ qua cả prefetch của trình duyệt như tài liệu Next.js (trang được prefetch sẽ không có CSP nào); thêm catch-all trong PR của DEC-113 (đổi phạm vi đã duyệt, STF-03 là màn hình admin kế tiếp).</t>
+        </is>
+      </c>
+      <c r="E115" s="2" t="inlineStr">
+        <is>
+          <t>Không đổi code: src/proxy.ts và docs/FRONTEND.md đã làm như (1) và (3) từ PR #85. PR web-only của STF-03 thêm catch-all của /admin kèm test Playwright (dòng STF-03 của docs/STATUS.md); web/CLAUDE.md ghi catch-all của /pos cho màn hình POS đầu tiên. docs/STATUS.md bỏ dòng Next dec-113-prefetch. Xem lại khi nâng Next.js mà cách prefetch hay trang 404 render động thay đổi.</t>
+        </is>
+      </c>
+      <c r="F115" s="2" t="inlineStr">
+        <is>
+          <t>Chủ dự án (các câu trả lời khi chạy PR #85, ngày 2026-10-22); DEC-113; PR #85 (Differences from DEC-113); web/src/proxy.ts; Next.js 16.4.2 docs: Content Security Policy</t>
+        </is>
+      </c>
+      <c r="G115" s="2" t="inlineStr">
+        <is>
+          <t>Phase 1</t>
+        </is>
+      </c>
+      <c r="H115" s="2" t="inlineStr">
+        <is>
+          <t>Accepted</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:H114"/>
+  <autoFilter ref="A1:H115"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
docs: record DEC-115 for web-only runs and web tests
DEC-115 aligns DEC-100 and DEC-110 with pull request #83 and the
pipeline: a done feature runs /implement-feature again for its
screens on feat/<id>-web, a second feat pull request and line of
issue #24; the test guide runs the Postman folder only when the API
changed and opens the screens with npm run dev, three manual checks
in all; and the jobs and required checks are those of pipeline.yml,
without a package or web-preview job.

docs/STATUS.md loses the row dec-web-run.

Refs: DEC-115, DEC-100, DEC-110
</commit_message>
<xml_diff>
--- a/docs/product-domain-blueprint-MVP.xlsx
+++ b/docs/product-domain-blueprint-MVP.xlsx
@@ -24,7 +24,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Use Cases'!$A$1:$L$140</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Domain Model'!$A$1:$J$78</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Business Rules'!$A$1:$I$137</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Decisions'!$A$1:$H$115</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Decisions'!$A$1:$H$116</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Technical Design'!$A$1:$E$17</definedName>
   </definedNames>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -30198,7 +30198,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H115"/>
+  <dimension ref="A1:H116"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -35041,8 +35041,50 @@
         </is>
       </c>
     </row>
+    <row r="116" ht="409.5" customHeight="1">
+      <c r="A116" s="3" t="inlineStr">
+        <is>
+          <t>DEC-115</t>
+        </is>
+      </c>
+      <c r="B116" s="2" t="inlineStr">
+        <is>
+          <t>Luồng web-only và kiểm thử có web</t>
+        </is>
+      </c>
+      <c r="C116" s="2" t="inlineStr">
+        <is>
+          <t>DEC-100 (1) cho mỗi tính năng một nhánh feat/&lt;id&gt; và một lần chạy; DEC-100 (3) cho hướng dẫn test trước merge chạy folder Postman của tính năng và tối đa 3 điểm kiểm tay; DEC-110 (1) coi một tính năng là xong khi PR feat của nó merge; DEC-100 (8) liệt kê job package, web-test và web-preview khi có web, và required checks PR gates, Validate PR title. Sau web-shell (PR #82), các màn hình SCR-AUT-02, SCR-ACC-01, SCR-STF-01 và SCR-STF-03 có API từ các tính năng đã xong (STF-03, STF-05, STF-02), nên ready check của /implement-feature dừng; chủ dự án chọn mỗi tính năng một PR màn hình qua /implement-feature thay vì viết prompt riêng cho từng màn hình. PR #83 thêm lần chạy web-only, chạy kiểm tra web và luồng Playwright trong /finish-feature và /fix-defect, và đổi hướng dẫn test. pipeline.yml hiện có: changes, secrets, tools-test, api-test, schema, web-test, acceptance (build image và migration bundle một lần, chạy toàn bộ collection Postman, trên main đẩy image lên GHCR, rồi chạy các luồng Playwright của web), ci-ok, deploy-staging, deploy-production; không có job package riêng hay web-preview; job được đặt tên trùng id nên required checks là ci-ok, pr-gates, pr-title. Đã so sánh: lần chạy web-only của /implement-feature; một prompt viết tay cho mỗi màn hình; giữ Postman ở mọi hướng dẫn test; chỉ chạy Postman khi API đổi.</t>
+        </is>
+      </c>
+      <c r="D116" s="2" t="inlineStr">
+        <is>
+          <t>(1) Sửa DEC-100 (1): một tính năng đã xong vẫn chạy được /implement-feature &lt;ID&gt; lần nữa khi docs/SCREENS.md mô tả một màn hình của nó có ô Blocked by trống mà web/ chưa có (route chưa có trang, hoặc còn trang tạm): lần chạy web-only chỉ làm các màn hình đó, không đổi API, migration hay collection Postman (cần thì là Needs decision), nhánh feat/&lt;id&gt;-web, và feat/&lt;id&gt;-web-2, -3… khi tên đó đã có PR merge, tiêu đề PR feat(web): &lt;subject&gt; (&lt;ID&gt;); /fix-defect không bị ràng buộc này. (2) Sửa DEC-110 (1): một tính năng xong khi PR feat đầu tiên của nó merge; mỗi lần chạy web-only sau đó là một PR feat nữa và một dòng nữa trong issue #24. (3) Sửa DEC-100 (3): hướng dẫn test trước merge chạy folder Postman của tính năng chỉ khi nhánh đổi api/ hoặc postman/; khi nhánh đổi web/, Claude để npm run dev chạy cạnh API và hướng dẫn mở màn hình ở http://localhost:3000; tổng số điểm kiểm tay, gồm cả màn hình, không quá 3; các luồng Playwright chạy ở /finish-feature bước 7 (sau toàn bộ collection) và trong job acceptance. (4) Sửa DEC-100 (8) theo pipeline.yml: các job changes, secrets, tools-test, api-test, schema, web-test, acceptance (gộp phần package: image và migration bundle build một lần, collection Postman, trên main đẩy GHCR, rồi các luồng Playwright), ci-ok, deploy-staging, deploy-production; không có job package riêng hay web-preview; tên job trùng id, required checks của main là ci-ok, pr-gates, pr-title. Không chọn: prompt viết tay cho mỗi màn hình (mỗi lần một prompt khác, không qua quy trình một lệnh của DEC-100 (2)); giữ Postman ở mọi hướng dẫn (thêm việc của chủ dự án khi API không đổi); job web-preview (deploy còn tắt tới khi có Vercel, ảnh chụp Playwright của acceptance thay thế cho hướng dẫn test).</t>
+        </is>
+      </c>
+      <c r="E116" s="2" t="inlineStr">
+        <is>
+          <t>Không đổi code: .claude/commands/implement-feature.md, finish-feature.md, fix-defect.md, docs/ACCEPTANCE.md và .github/workflows/pipeline.yml đã làm như (1) tới (4) từ PR #83 và các PR công cụ. Mỗi màn hình của một tính năng đã xong thêm một PR feat(web) và một dòng issue #24 có cùng Feature ID; routine ZenGear PR merged không đổi (mục (4) của dòng Waiting về DEC-112 kiểm cách nó đếm kịch bản). docs/STATUS.md bỏ dòng Next dec-web-run. Xem lại khi bật deploy lên Vercel (web-preview) hoặc khi lần chạy web-only đầu tiên (STF-03) cho thấy ready check cần đổi.</t>
+        </is>
+      </c>
+      <c r="F116" s="2" t="inlineStr">
+        <is>
+          <t>Chủ dự án (các lựa chọn ngày 2026-10-21 và 2026-10-22); DEC-100; DEC-104 (8); DEC-110; PR #82; PR #83 (Differences from accepted Decisions, Decisions made); .claude/commands/implement-feature.md; .claude/commands/finish-feature.md; .github/workflows/pipeline.yml</t>
+        </is>
+      </c>
+      <c r="G116" s="2" t="inlineStr">
+        <is>
+          <t>Phase 1</t>
+        </is>
+      </c>
+      <c r="H116" s="2" t="inlineStr">
+        <is>
+          <t>Accepted</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:H115"/>
+  <autoFilter ref="A1:H116"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>